<commit_message>
Corrección plantillas Aut Dev
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/AutDev-CuentasCuentasSeguidas-2706.xlsx
+++ b/public/CuentasCuentas/AutDev-CuentasCuentasSeguidas-2706.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\CuentasCuentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B62438-B9A8-489D-BCA3-0464E89AA2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF0D10C-AFB4-4067-B5AF-ED4E0A5D6F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="72">
   <si>
     <t>cuenta</t>
   </si>
@@ -246,6 +246,12 @@
   </si>
   <si>
     <t>Por la autorización de la devolución de ingresos de aportaciones. 1</t>
+  </si>
+  <si>
+    <t>II.1.8 PARTICIPACIONES, APORTACIONES, CONVENIOS, INCENTIVOS DERIVADOS DE LA COLABORACIÓN FISCAL, FONDOS DISTINTOS DE APORTACIONES, TRANSFERENCIAS, ASIGNACIONES, SUBSIDIOS Y SUBVENCIONES, Y PENSIONES Y JUBILACIONES</t>
+  </si>
+  <si>
+    <t>II.1.7.1 VENTA DE BIENES Y PRESTACIÓN DE SERVICIOS (VENTAS)</t>
   </si>
 </sst>
 </file>
@@ -809,7 +815,7 @@
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
         <v>47</v>
@@ -823,7 +829,7 @@
         <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -837,7 +843,7 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
         <v>47</v>
@@ -851,7 +857,7 @@
         <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -865,7 +871,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
         <v>47</v>
@@ -879,7 +885,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
         <v>47</v>
@@ -893,7 +899,7 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -907,7 +913,7 @@
         <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
         <v>53</v>
@@ -921,7 +927,7 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
         <v>53</v>
@@ -935,7 +941,7 @@
         <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>53</v>
@@ -949,7 +955,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C24" t="s">
         <v>53</v>
@@ -963,7 +969,7 @@
         <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
         <v>53</v>
@@ -977,7 +983,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
         <v>53</v>
@@ -991,7 +997,7 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s">
         <v>53</v>
@@ -1005,7 +1011,7 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C28" t="s">
         <v>53</v>
@@ -1019,7 +1025,7 @@
         <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C29" t="s">
         <v>53</v>
@@ -1033,7 +1039,7 @@
         <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C30" t="s">
         <v>53</v>
@@ -1047,7 +1053,7 @@
         <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C31" t="s">
         <v>53</v>
@@ -1061,7 +1067,7 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
         <v>53</v>
@@ -1075,7 +1081,7 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C33" t="s">
         <v>53</v>
@@ -1089,7 +1095,7 @@
         <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C34" t="s">
         <v>53</v>
@@ -1103,7 +1109,7 @@
         <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C35" t="s">
         <v>53</v>
@@ -1117,7 +1123,7 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C36" t="s">
         <v>53</v>
@@ -1131,7 +1137,7 @@
         <v>56</v>
       </c>
       <c r="B37" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C37" t="s">
         <v>53</v>
@@ -1145,7 +1151,7 @@
         <v>25</v>
       </c>
       <c r="B38" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C38" t="s">
         <v>53</v>
@@ -1159,7 +1165,7 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C39" t="s">
         <v>53</v>
@@ -1173,7 +1179,7 @@
         <v>25</v>
       </c>
       <c r="B40" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C40" t="s">
         <v>53</v>
@@ -1187,7 +1193,7 @@
         <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C41" t="s">
         <v>53</v>
@@ -1201,7 +1207,7 @@
         <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
         <v>53</v>
@@ -1215,7 +1221,7 @@
         <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
         <v>53</v>
@@ -1229,7 +1235,7 @@
         <v>26</v>
       </c>
       <c r="B44" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C44" t="s">
         <v>53</v>
@@ -1243,7 +1249,7 @@
         <v>57</v>
       </c>
       <c r="B45" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C45" t="s">
         <v>53</v>
@@ -1257,7 +1263,7 @@
         <v>26</v>
       </c>
       <c r="B46" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C46" t="s">
         <v>53</v>
@@ -1271,7 +1277,7 @@
         <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C47" t="s">
         <v>53</v>
@@ -1285,7 +1291,7 @@
         <v>27</v>
       </c>
       <c r="B48" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C48" t="s">
         <v>53</v>
@@ -1299,7 +1305,7 @@
         <v>13</v>
       </c>
       <c r="B49" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C49" t="s">
         <v>53</v>
@@ -1313,7 +1319,7 @@
         <v>27</v>
       </c>
       <c r="B50" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
         <v>53</v>
@@ -1327,7 +1333,7 @@
         <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C51" t="s">
         <v>53</v>
@@ -1341,7 +1347,7 @@
         <v>27</v>
       </c>
       <c r="B52" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C52" t="s">
         <v>53</v>
@@ -1355,7 +1361,7 @@
         <v>41</v>
       </c>
       <c r="B53" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C53" t="s">
         <v>53</v>
@@ -1369,7 +1375,7 @@
         <v>27</v>
       </c>
       <c r="B54" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C54" t="s">
         <v>53</v>
@@ -1383,7 +1389,7 @@
         <v>38</v>
       </c>
       <c r="B55" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="C55" t="s">
         <v>53</v>
@@ -1397,7 +1403,7 @@
         <v>28</v>
       </c>
       <c r="B56" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C56" t="s">
         <v>53</v>
@@ -1411,7 +1417,7 @@
         <v>14</v>
       </c>
       <c r="B57" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C57" t="s">
         <v>53</v>
@@ -1425,7 +1431,7 @@
         <v>28</v>
       </c>
       <c r="B58" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C58" t="s">
         <v>53</v>
@@ -1439,7 +1445,7 @@
         <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C59" t="s">
         <v>53</v>
@@ -1453,7 +1459,7 @@
         <v>28</v>
       </c>
       <c r="B60" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C60" t="s">
         <v>53</v>
@@ -1467,7 +1473,7 @@
         <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C61" t="s">
         <v>53</v>
@@ -1481,7 +1487,7 @@
         <v>29</v>
       </c>
       <c r="B62" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C62" t="s">
         <v>53</v>
@@ -1495,7 +1501,7 @@
         <v>15</v>
       </c>
       <c r="B63" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C63" t="s">
         <v>53</v>
@@ -1509,7 +1515,7 @@
         <v>29</v>
       </c>
       <c r="B64" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C64" t="s">
         <v>53</v>
@@ -1523,7 +1529,7 @@
         <v>60</v>
       </c>
       <c r="B65" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C65" t="s">
         <v>53</v>
@@ -1537,7 +1543,7 @@
         <v>29</v>
       </c>
       <c r="B66" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C66" t="s">
         <v>53</v>
@@ -1551,7 +1557,7 @@
         <v>43</v>
       </c>
       <c r="B67" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C67" t="s">
         <v>53</v>
@@ -1565,7 +1571,7 @@
         <v>29</v>
       </c>
       <c r="B68" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C68" t="s">
         <v>53</v>
@@ -1579,7 +1585,7 @@
         <v>38</v>
       </c>
       <c r="B69" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C69" t="s">
         <v>53</v>
@@ -1593,7 +1599,7 @@
         <v>30</v>
       </c>
       <c r="B70" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C70" t="s">
         <v>53</v>
@@ -1607,7 +1613,7 @@
         <v>16</v>
       </c>
       <c r="B71" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C71" t="s">
         <v>53</v>
@@ -1621,7 +1627,7 @@
         <v>30</v>
       </c>
       <c r="B72" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C72" t="s">
         <v>53</v>
@@ -1635,7 +1641,7 @@
         <v>61</v>
       </c>
       <c r="B73" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C73" t="s">
         <v>53</v>
@@ -1649,7 +1655,7 @@
         <v>30</v>
       </c>
       <c r="B74" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C74" t="s">
         <v>53</v>
@@ -1663,7 +1669,7 @@
         <v>44</v>
       </c>
       <c r="B75" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C75" t="s">
         <v>53</v>
@@ -1677,7 +1683,7 @@
         <v>30</v>
       </c>
       <c r="B76" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C76" t="s">
         <v>53</v>
@@ -1691,7 +1697,7 @@
         <v>38</v>
       </c>
       <c r="B77" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C77" t="s">
         <v>53</v>
@@ -1705,7 +1711,7 @@
         <v>31</v>
       </c>
       <c r="B78" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C78" t="s">
         <v>53</v>
@@ -1719,7 +1725,7 @@
         <v>17</v>
       </c>
       <c r="B79" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C79" t="s">
         <v>53</v>
@@ -1733,7 +1739,7 @@
         <v>31</v>
       </c>
       <c r="B80" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C80" t="s">
         <v>53</v>
@@ -1747,7 +1753,7 @@
         <v>62</v>
       </c>
       <c r="B81" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C81" t="s">
         <v>53</v>
@@ -1761,7 +1767,7 @@
         <v>31</v>
       </c>
       <c r="B82" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C82" t="s">
         <v>53</v>
@@ -1775,7 +1781,7 @@
         <v>45</v>
       </c>
       <c r="B83" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C83" t="s">
         <v>53</v>
@@ -1789,7 +1795,7 @@
         <v>31</v>
       </c>
       <c r="B84" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C84" t="s">
         <v>53</v>
@@ -1803,7 +1809,7 @@
         <v>38</v>
       </c>
       <c r="B85" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C85" t="s">
         <v>53</v>

</xml_diff>